<commit_message>
Document polish: fix Generated date on page 1, widen xlsx Summary label column
</commit_message>
<xml_diff>
--- a/generated-docs/Nof1_FormulationSchedule_SUB-2026-003_DRAFT.xlsx
+++ b/generated-docs/Nof1_FormulationSchedule_SUB-2026-003_DRAFT.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="178">
   <si>
     <t>W Code</t>
   </si>
@@ -50,49 +50,142 @@
     <t>Evidence Pointer</t>
   </si>
   <si>
+    <t>W140010000</t>
+  </si>
+  <si>
+    <t>N-acetyl cysteine (NAC)</t>
+  </si>
+  <si>
+    <t>mg</t>
+  </si>
+  <si>
+    <t>Antioxidant / Redox</t>
+  </si>
+  <si>
+    <t>STANDARD</t>
+  </si>
+  <si>
+    <t>8-OHdG 3.80, Pyroglutamic 28.8, t,t-Muconic 0.20</t>
+  </si>
+  <si>
+    <t>Glutathione precursor supporting xenobiotic conjugation and antioxidant defence; addresses 8-OHdG 3.80 (&lt;2.70), pyroglutamic acid at upper range, and the xenobiotic burden pattern (t,t-muconic, 3-methylhippuric).</t>
+  </si>
+  <si>
+    <t>Standard contraindication checks: medications not listed in submission; NAC is generally well tolerated.</t>
+  </si>
+  <si>
+    <t>Published evidence supports NAC for glutathione repletion and antioxidant support; clinical relevance for this patient is for practitioner assessment.</t>
+  </si>
+  <si>
+    <t>W010013000</t>
+  </si>
+  <si>
+    <t>Milk thistle (silymarin)</t>
+  </si>
+  <si>
+    <t>Heavy Metal Detox</t>
+  </si>
+  <si>
+    <t>t,t-Muconic 0.20, 5-HMF 18.5, Benzoic 25.0</t>
+  </si>
+  <si>
+    <t>Nrf2-mediated Phase II upregulation and hepatoprotection; addresses xenobiotic-burdened pattern (t,t-muconic, 3-methylhippuric, 4-HBA, 5-HMF).</t>
+  </si>
+  <si>
+    <t>Generally well tolerated.</t>
+  </si>
+  <si>
+    <t>Published mechanism and clinical literature supports milk thistle as hepatic/Phase II support — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W040012000</t>
+  </si>
+  <si>
+    <t>Calcium D-glucarate</t>
+  </si>
+  <si>
+    <t>4-HBA 0.64, 5-HMF 18.5, Benzoic 25.0</t>
+  </si>
+  <si>
+    <t>Glucuronidation support via beta-glucuronidase inhibition; addresses paraben/phthalate/xenobiotic conjugation load.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; phthalate marker within range but paraben (4-HBA) elevated.</t>
+  </si>
+  <si>
+    <t>Published mechanism literature supports Cal D-glucarate for Phase II glucuronidation — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W030001000</t>
+  </si>
+  <si>
+    <t>Vitamin C (ascorbic acid)</t>
+  </si>
+  <si>
+    <t>8-OHdG 3.80</t>
+  </si>
+  <si>
+    <t>Antioxidant defence aligned with elevated 8-OHdG and broad xenobiotic redox demand.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; consider divided doses if GI tolerability is an issue.</t>
+  </si>
+  <si>
+    <t>Published evidence supports vitamin C as a water-soluble antioxidant — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W010019000</t>
+  </si>
+  <si>
+    <t>Resveratrol</t>
+  </si>
+  <si>
+    <t>8-OHdG 3.80, LTE4 195</t>
+  </si>
+  <si>
+    <t>Nrf2/sirtuin antioxidant support complementing NAC and vitamin C for the oxidative stress pattern.</t>
+  </si>
+  <si>
+    <t>Anticoagulant interaction theoretical; practitioner to review medications.</t>
+  </si>
+  <si>
+    <t>Published RCT and mechanism literature for antioxidant/anti-inflammatory effects — practitioner to assess.</t>
+  </si>
+  <si>
     <t>W010029000</t>
   </si>
   <si>
     <t>Turmeric (curcumin)</t>
   </si>
   <si>
-    <t>mg</t>
-  </si>
-  <si>
     <t>Anti-inflammatory Core</t>
   </si>
   <si>
-    <t>STANDARD</t>
-  </si>
-  <si>
-    <t>Leukotriene E4 195 (H), 8-OHdG 3.80 (H), Quinolinic 11.80 (H)</t>
-  </si>
-  <si>
-    <t>Curcumin (turmeric 25:1 extract, 40% curcuminoids) as the NF-κB-directed anti-inflammatory anchor for the inflammatory pattern (Leukotriene E4 195 H, 8-OHdG 3.80 H, kynurenine-pathway shunt). Dose at ~75% of the Library maximum (1000 mg) per published RCT ranges for systemic inflammation support.</t>
-  </si>
-  <si>
-    <t>Use with caution alongside anticoagulants; published reports note rare hepatic adverse events.</t>
-  </si>
-  <si>
-    <t>RCT and meta-analysis evidence for curcumin in chronic inflammation and CRP reduction; see Library references list.</t>
+    <t>LTE4 195, Quinolinic 11.8</t>
+  </si>
+  <si>
+    <t>NF-κB anchor for inflammatory load (LTE4 elevation, kynurenine inflammatory shift).</t>
+  </si>
+  <si>
+    <t>Caution with anticoagulants; standard contraindication checks.</t>
+  </si>
+  <si>
+    <t>RCT evidence supports curcumin's anti-inflammatory mechanism — practitioner to assess.</t>
   </si>
   <si>
     <t>W010022000</t>
   </si>
   <si>
-    <t>Boswellia (frankincense)</t>
-  </si>
-  <si>
-    <t>Leukotriene E4 195 (H)</t>
-  </si>
-  <si>
-    <t>Boswellia 6:1 (60% boswellic acids) — 5-LOX-inhibitor mechanism is directly relevant to the elevated Leukotriene E4. Layer-dose at ~25% of clinical target (recommended 800 mg) to fit budget; original target 800 mg.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; mild GI effects possible.</t>
-  </si>
-  <si>
-    <t>Boswellic acids inhibit 5-LOX; clinical trials in inflammatory conditions support consideration.</t>
+    <t>Boswellia serrata</t>
+  </si>
+  <si>
+    <t>LTE4 195</t>
+  </si>
+  <si>
+    <t>5-LOX inhibition specifically relevant to elevated leukotriene E4. Dose trimmed for pod budget; clinical target 800 mg may be considered as additional standalone if indicated.</t>
+  </si>
+  <si>
+    <t>Published evidence for 5-LOX-pathway modulation — practitioner to assess.</t>
   </si>
   <si>
     <t>W010031000</t>
@@ -101,109 +194,10 @@
     <t>Quercetin</t>
   </si>
   <si>
-    <t>Leukotriene E4 195 (H), 8-OHdG 3.80 (H)</t>
-  </si>
-  <si>
-    <t>Quercetin as an anti-inflammatory / antioxidant layer with mast-cell-stabilising activity, complementing curcumin and boswellia.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; high doses may cause headache or tingling.</t>
-  </si>
-  <si>
-    <t>Quercetin RCT evidence for anti-inflammatory and antihypertensive effects.</t>
-  </si>
-  <si>
-    <t>W010019000</t>
-  </si>
-  <si>
-    <t>Resveratrol</t>
-  </si>
-  <si>
-    <t>8-OHdG 3.80 (H), Mevalonolactone 2.80 (H)</t>
-  </si>
-  <si>
-    <t>Trans-resveratrol at the Library/regulatory maximum (150 mg) for Nrf2/SIRT pathway support and antioxidant cover for the elevated 8-OHdG.</t>
-  </si>
-  <si>
-    <t>May affect coagulation — caution with anticoagulants.</t>
-  </si>
-  <si>
-    <t>RCT evidence for resveratrol on glucose, vascular and antioxidant endpoints.</t>
-  </si>
-  <si>
-    <t>W140010000</t>
-  </si>
-  <si>
-    <t>N-acetyl cysteine (NAC)</t>
-  </si>
-  <si>
-    <t>Antioxidant / Redox</t>
-  </si>
-  <si>
-    <t>t,t-Muconic 0.20 (H), Pyroglutamic 28.8 (top of range), 8-OHdG 3.80 (H)</t>
-  </si>
-  <si>
-    <t>NAC as the glutathione precursor foundational for xenobiotic Phase II support given the benzene/xylene/paraben pattern (t,t-muconic, 3-methylhippuric, 4-HBA) and pyroglutamic at the top of range (glutathione cycling pressure).</t>
-  </si>
-  <si>
-    <t>GI effects possible; uncommon allergic reactions.</t>
-  </si>
-  <si>
-    <t>RCT evidence for NAC supporting glutathione status and respiratory/oxidative outcomes.</t>
-  </si>
-  <si>
-    <t>W010013000</t>
-  </si>
-  <si>
-    <t>Milk thistle (silymarin)</t>
-  </si>
-  <si>
-    <t>t,t-Muconic 0.20 (H), 4-HBA 0.64 (H), 8-OHdG 3.80 (H)</t>
-  </si>
-  <si>
-    <t>Silymarin as Nrf2-mediated Phase II upregulator and hepatic support given xenobiotic load. Dose at recommended 150 mg.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; mild GI effects.</t>
-  </si>
-  <si>
-    <t>Silymarin clinical evidence in hepatic and Phase II contexts.</t>
-  </si>
-  <si>
-    <t>W040012000</t>
-  </si>
-  <si>
-    <t>Calcium D-glucarate</t>
-  </si>
-  <si>
-    <t>4-HBA 0.64 (H), Benzoic 25.0 (H), t,t-Muconic 0.20 (H)</t>
-  </si>
-  <si>
-    <t>Calcium D-glucarate supports glucuronidation Phase II conjugation — directly relevant to the paraben (4-HBA) and benzoate-conjugation pattern.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated.</t>
-  </si>
-  <si>
-    <t>Published reviews of calcium D-glucarate in beta-glucuronidase modulation and xenobiotic clearance.</t>
-  </si>
-  <si>
-    <t>W030001000</t>
-  </si>
-  <si>
-    <t>Vitamin C (ascorbic acid)</t>
-  </si>
-  <si>
-    <t>8-OHdG 3.80 (H), t,t-Muconic 0.20 (H)</t>
-  </si>
-  <si>
-    <t>Aqueous antioxidant cover given elevated 8-OHdG and xenobiotic load; supports collagen integrity and immune function.</t>
-  </si>
-  <si>
-    <t>High doses can cause GI upset; caution with haemochromatosis.</t>
-  </si>
-  <si>
-    <t>Established literature on vitamin C and oxidative stress.</t>
+    <t>Mast-cell stabilising and adjunctive anti-inflammatory action complementing LTE4-driven inflammation.</t>
+  </si>
+  <si>
+    <t>Published mechanism literature for mast-cell modulation — practitioner to assess.</t>
   </si>
   <si>
     <t>W030021000</t>
@@ -215,16 +209,16 @@
     <t>Mitochondrial / Cardiovascular</t>
   </si>
   <si>
-    <t>Mevalonolactone 2.80 (H), Isocitric 86 (H), 2-Oxoglutaric 65 (H)</t>
-  </si>
-  <si>
-    <t>CoQ10 100 mg foundational mitochondrial electron transport support given elevated mevalonolactone (HMG-CoA reductase activity) and TCA accumulation pattern.</t>
-  </si>
-  <si>
-    <t>May interact with warfarin.</t>
-  </si>
-  <si>
-    <t>RCT evidence for CoQ10 in cardiovascular and mitochondrial contexts.</t>
+    <t>3-MGA 6.32, Mevalonolactone 2.80, Isocitrate 86, 2-OG 65</t>
+  </si>
+  <si>
+    <t>Mitochondrial electron transport and mevalonate pathway support; addresses 3-MGA, mevalonolactone, and TCA cycle markers.</t>
+  </si>
+  <si>
+    <t>Standard interaction note with warfarin.</t>
+  </si>
+  <si>
+    <t>Published cardiology/mitochondrial literature — practitioner to assess.</t>
   </si>
   <si>
     <t>W030020000</t>
@@ -233,148 +227,133 @@
     <t>Alpha-lipoic acid</t>
   </si>
   <si>
-    <t>2-Oxoglutaric 65 (H), Isocitric 86 (H), 8-OHdG 3.80 (H)</t>
-  </si>
-  <si>
-    <t>ALA at 150 mg — cofactor for α-KGDH and pyruvate dehydrogenase, redox-active. Directly relevant to elevated 2-oxoglutaric. Original target 300 mg; reduced to fit budget.</t>
-  </si>
-  <si>
-    <t>May lower blood glucose.</t>
-  </si>
-  <si>
-    <t>RCT evidence for ALA in glycaemic and antioxidant contexts.</t>
+    <t>2-OG 65, Isocitrate 86, 8-OHdG 3.80</t>
+  </si>
+  <si>
+    <t>Cofactor for 2-OG dehydrogenase and pyruvate dehydrogenase; addresses 2-OG and isocitrate elevation and contributes to antioxidant defence.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; mild hypoglycaemic effect possible.</t>
+  </si>
+  <si>
+    <t>Published mechanism literature — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W030008000</t>
+  </si>
+  <si>
+    <t>Methylcobalamin (B12)</t>
+  </si>
+  <si>
+    <t>mcg</t>
+  </si>
+  <si>
+    <t>B-Vitamins / Methylation</t>
+  </si>
+  <si>
+    <t>Guanidinoacetic 4.80, KMBA 3.20, 5-Methylcytosine 68</t>
+  </si>
+  <si>
+    <t>Methylation cycle support addressing methyl-acceptor demand (guanidinoacetic, KMBA, 5-methylcytosine).</t>
+  </si>
+  <si>
+    <t>Standard B12 considerations.</t>
+  </si>
+  <si>
+    <t>Published methylation literature — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W030027000</t>
+  </si>
+  <si>
+    <t>Calcium folinate</t>
+  </si>
+  <si>
+    <t>Guanidinoacetic 4.80, 5-Methylcytosine 68</t>
+  </si>
+  <si>
+    <t>Folate cycle cofactor for one-carbon metabolism; supports the methylation demand pattern.</t>
+  </si>
+  <si>
+    <t>May mask B12 deficiency in megaloblastic anaemia — B12 included concurrently.</t>
   </si>
   <si>
     <t>W030012000</t>
   </si>
   <si>
-    <t>Vitamin B6 (pyridoxal 5-phosphate)</t>
-  </si>
-  <si>
-    <t>B-Vitamins / Methylation</t>
-  </si>
-  <si>
-    <t>MODERATE</t>
-  </si>
-  <si>
-    <t>Xanthurenic 1.92 (H), Kynurenic 3.10 (H)</t>
-  </si>
-  <si>
-    <t>P5P 15 mg (delivers ~10 mg pyridoxine equivalent) as the foundational B6 input for kynurenine pathway redirection — xanthurenic elevation indicates functional B6 demand. Dose set below 50 mg/day caution threshold for peripheral neuropathy.</t>
-  </si>
-  <si>
-    <t>TGA warning on B6 — stop and review if tingling/numbness; total daily B6 from all sources should be monitored.</t>
-  </si>
-  <si>
-    <t>Published frameworks linking xanthurenic acid elevation to B6-dependent kynurenine pathway flux.</t>
-  </si>
-  <si>
-    <t>W030008000</t>
-  </si>
-  <si>
-    <t>Vitamin B12 (methylcobalamin)</t>
-  </si>
-  <si>
-    <t>mcg</t>
-  </si>
-  <si>
-    <t>KMBA 3.20 (H), Guanidinoacetic 4.80 (H)</t>
-  </si>
-  <si>
-    <t>Methylcobalamin 500 mcg supports methyl pool given KMBA elevation (methionine metabolism), guanidinoacetic acid elevation (creatine methylation demand) and the 5-methylcytosine elevation pattern.</t>
-  </si>
-  <si>
-    <t>Standard B12 dosing for methylation cofactor support.</t>
+    <t>Pyridoxal-5-phosphate (P5P / active B6)</t>
+  </si>
+  <si>
+    <t>Xanthurenic 1.92, Quinolinic 11.8, Kynurenic 3.10</t>
+  </si>
+  <si>
+    <t>Active B6 anchoring kynurenine pathway support given xanthurenic 1.92 (&lt;0.96) and quinolinic 11.8 (&lt;9.10); B6 cofactor for kynureninase.</t>
+  </si>
+  <si>
+    <t>TGA advises stopping if tingling/numbness occurs; dose kept conservative.</t>
+  </si>
+  <si>
+    <t>Published kynurenine pathway literature — practitioner to assess.</t>
   </si>
   <si>
     <t>W030011000</t>
   </si>
   <si>
-    <t>Vitamin B2 (riboflavin)</t>
-  </si>
-  <si>
-    <t>2-Oxoglutaric 65 (H), Xanthurenic 1.92 (H)</t>
-  </si>
-  <si>
-    <t>Riboflavin 20 mg — FAD cofactor for α-KGDH complex (directly relevant to elevated 2-oxoglutaric) and for B6 activation to P5P.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; benign yellow urine colour expected.</t>
-  </si>
-  <si>
-    <t>Established role of riboflavin in α-KGDH and B6 activation.</t>
-  </si>
-  <si>
-    <t>W030009000</t>
-  </si>
-  <si>
-    <t>Folate (calcium levomefolate)</t>
-  </si>
-  <si>
-    <t>L-5-MTHF 520 mcg (delivers ~400 mcg levomefolic acid equivalent) — methylation cofactor partner for B12, given KMBA and guanidinoacetic elevation. Dose within TGA limit.</t>
-  </si>
-  <si>
-    <t>Caution with high-dose folate masking B12 deficiency — co-administered here.</t>
-  </si>
-  <si>
-    <t>Published evidence for methylfolate in methylation support.</t>
-  </si>
-  <si>
-    <t>W010026000</t>
-  </si>
-  <si>
-    <t>Berberine HCl</t>
-  </si>
-  <si>
-    <t>Gastrointestinal</t>
-  </si>
-  <si>
-    <t>Arabinose 42 (H), 3,4-DHBA 62 (H), Furancarbonylglycine 2.90 (H)</t>
-  </si>
-  <si>
-    <t>Berberine 500 mg as gastrointestinal axis support for the dysbiosis fingerprint (arabinose, microbial polyphenol metabolites, furan derivatives). Also has favourable metabolic profile.</t>
-  </si>
-  <si>
-    <t>Avoid in pregnancy; potential CYP interactions; may lower blood glucose.</t>
-  </si>
-  <si>
-    <t>RCT evidence for berberine in metabolic and antimicrobial contexts.</t>
-  </si>
-  <si>
-    <t>W140005000</t>
-  </si>
-  <si>
-    <t>L-glutamine</t>
-  </si>
-  <si>
-    <t>Arabinose 42 (H), Dysbiosis fingerprint</t>
-  </si>
-  <si>
-    <t>L-glutamine at modest in-pod dose for gut barrier support alongside the dysbiosis fingerprint. Clinical target dose for IBS/barrier support is 3-5 g daily — surfaced as standalone for higher dose; in-pod dose at 200 mg is supportive only.</t>
-  </si>
-  <si>
-    <t>RCT evidence for L-glutamine in gut barrier/IBS contexts.</t>
-  </si>
-  <si>
-    <t>W040008000</t>
-  </si>
-  <si>
-    <t>Zinc citrate</t>
+    <t>Riboflavin (B2)</t>
+  </si>
+  <si>
+    <t>2-OG 65, Kynurenic 3.10</t>
+  </si>
+  <si>
+    <t>FAD cofactor for mitochondrial flavoproteins and kynurenine monooxygenase; supports both TCA strain and kynurenine pattern.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; yellow urine expected.</t>
+  </si>
+  <si>
+    <t>Published B2 metabolism literature — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W040002000</t>
+  </si>
+  <si>
+    <t>Magnesium glycinate</t>
   </si>
   <si>
     <t>Minerals</t>
   </si>
   <si>
-    <t>Broad cofactor support</t>
-  </si>
-  <si>
-    <t>Zinc citrate delivering ~25 mg elemental zinc for broad cofactor support and immune/IDO-axis context. Within AUST L cap.</t>
-  </si>
-  <si>
-    <t>Long-term zinc supplementation (&gt;3 months) may affect copper status — practitioner to monitor.</t>
-  </si>
-  <si>
-    <t>Established zinc supplementation evidence.</t>
+    <t>2-OG 65, Isocitrate 86, Guanidinoacetic 4.80</t>
+  </si>
+  <si>
+    <t>Broad mitochondrial/methylation cofactor at conservative in-pod elemental dose (100 mg). The glycinate carrier also contributes glycine equivalents incidentally supportive of conjugation pathways. Practitioner may wish to consider additional standalone magnesium toward a clinical target if symptomatically indicated.</t>
+  </si>
+  <si>
+    <t>Standard renal considerations.</t>
+  </si>
+  <si>
+    <t>Published magnesium clinical literature — practitioner to assess.</t>
+  </si>
+  <si>
+    <t>W030005000</t>
+  </si>
+  <si>
+    <t>Vitamin D3 (cholecalciferol)</t>
+  </si>
+  <si>
+    <t>Vitamin D / C / Neurotransmitter</t>
+  </si>
+  <si>
+    <t>General repletion</t>
+  </si>
+  <si>
+    <t>Conservative repletion dose at AUST L cap (25 mcg = 1000 IU); supports general immune/redox status. 25-OH D not measured on this panel.</t>
+  </si>
+  <si>
+    <t>Practitioner may wish to assess serum 25-OH D to guide longer-term dosing.</t>
+  </si>
+  <si>
+    <t>Published vitamin D supplementation literature — practitioner to assess.</t>
   </si>
   <si>
     <t>Adjustment Type</t>
@@ -386,25 +365,16 @@
     <t>Affected Ingredient(s)</t>
   </si>
   <si>
-    <t>reduced_for_budget</t>
-  </si>
-  <si>
-    <t>Boswellia reduced from a clinical target of 800 mg to 200 mg to fit the pod-budget; the practitioner may wish to consider a higher dose if clinically indicated (boswellia is a high-loading-cost ingredient at 5 mg/granule).</t>
+    <t>in_pod_dose_below_clinical_target</t>
+  </si>
+  <si>
+    <t>Boswellia in-pod dose 300 mg vs clinical target 800 mg — trimmed for pod budget. Practitioner may consider standalone top-up.</t>
   </si>
   <si>
     <t>Boswellia (Frankincense)</t>
   </si>
   <si>
-    <t>Alpha-lipoic acid reduced from a 300 mg target to 150 mg to balance pod budget across axes.</t>
-  </si>
-  <si>
-    <t>R,S-alpha lipoic acid</t>
-  </si>
-  <si>
-    <t>in_pod_supportive_dose</t>
-  </si>
-  <si>
-    <t>L-glutamine 200 mg in-pod is supportive only; clinical target for gut barrier support is 3-5 g daily and would need to be delivered standalone if clinically indicated.</t>
+    <t>Magnesium glycinate in-pod elemental 100 mg vs broader clinical target — split-dosing may be considered.</t>
   </si>
   <si>
     <t>Recommendation</t>
@@ -416,34 +386,31 @@
     <t>Practitioner Note</t>
   </si>
   <si>
-    <t>Glycine 1-3 g daily</t>
+    <t>Glycine 1.5–3 g daily</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Glycine is the canonical Phase II conjugator for benzoate and xylene metabolites and is not in the current Library. The practitioner may wish to consider standalone glycine supplementation given elevated benzoic acid and 3-methylhippuric acid.</t>
-  </si>
-  <si>
-    <t>EPA/DHA fish oil 2-3 g daily</t>
-  </si>
-  <si>
-    <t>Omega-3 fatty acids may complement the anti-inflammatory stack by modulating leukotriene pathway flux; not in the current Library.</t>
-  </si>
-  <si>
-    <t>Multi-strain probiotic (Lactobacillus and Bifidobacterium spp., 20-40 billion CFU)</t>
-  </si>
-  <si>
-    <t>Targeted probiotic support may complement berberine for the dysbiosis fingerprint; not available in the current granule Library.</t>
-  </si>
-  <si>
-    <t>5-HTP (excluded from pod: deprioritised)</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Low 5-HIAA alongside elevated quinolinic suggests reduced serotonin pathway throughput per published frameworks. 5-HTP has not been included in the pod pending practitioner review of medication context — published literature warns of serotonin syndrome risk with concurrent serotonergic medications (SSRIs/SNRIs/MAOIs/tricyclics/triptans/tramadol). Practitioner may wish to consider 50-100 mg daily standalone once medication context is confirmed.</t>
+    <t>Glycine is the canonical Phase II conjugator for benzoate, xylene/toluene metabolites and HMF-derived furancarbonyl conjugates. Given elevated benzoic acid, 3-methylhippuric, 4-HBA and furancarbonylglycine, the practitioner may wish to consider glycine repletion alongside the in-pod conjugation support. Not in current Library as a granule ingredient.</t>
+  </si>
+  <si>
+    <t>EPA/DHA omega-3 fish oil 2–3 g daily</t>
+  </si>
+  <si>
+    <t>Given leukotriene E4 elevation (195 vs &lt;100), the practitioner may wish to consider an EPA-predominant omega-3 to shift eicosanoid balance. Not in current granule Library.</t>
+  </si>
+  <si>
+    <t>L-carnitine 1–2 g daily</t>
+  </si>
+  <si>
+    <t>Given mild adipic acid elevation suggesting omega-oxidation when beta-oxidation is constrained, the practitioner may wish to consider carnitine support. Not in current Library.</t>
+  </si>
+  <si>
+    <t>Multi-strain probiotic (Lactobacillus / Bifidobacterium spp.) 20–40 billion CFU daily</t>
+  </si>
+  <si>
+    <t>Given modest dysbiosis markers (arabinose, 3,4-DHBA, 3-HPAA), the practitioner may wish to consider probiotic support and dietary review. Not in current granule Library.</t>
   </si>
   <si>
     <t>Severity</t>
@@ -455,37 +422,59 @@
     <t>informational</t>
   </si>
   <si>
-    <t>medication_context_not_provided</t>
-  </si>
-  <si>
-    <t>No medication list was supplied with the submission. Standard checks have been run against the proposed ingredients alone. Specifically: 5-HTP excluded pending serotonergic medication review; curcumin and resveratrol carry bleeding-risk caveats with anticoagulants; berberine has CYP3A4/CYP2D6 interaction potential and additive glucose-lowering risk; vitamin C caution with haemochromatosis.</t>
+    <t>no_medication_list_provided</t>
+  </si>
+  <si>
+    <t>Clinical notes did not list current medications. Standard contraindication screens (5-HTP with serotonergics; berberine with glucose-lowering agents; curcumin/resveratrol with anticoagulants; magnesium with antibiotics/bisphosphonates; St John's Wort with multiple meds) were therefore applied to the formulation in the abstract. 5-HTP and berberine were not included in this formulation. Curcumin, resveratrol and magnesium have been included — practitioner to verify against the patient's full medication list.</t>
   </si>
   <si>
     <t>—</t>
   </si>
   <si>
-    <t>monitor</t>
-  </si>
-  <si>
-    <t>B6_neuropathy_monitoring</t>
-  </si>
-  <si>
-    <t>P5P 15 mg supplied in pod is well below the 50 mg neuropathy-caution threshold, but practitioner should be aware of cumulative B6 intake from all sources and review for any sensory symptoms.</t>
-  </si>
-  <si>
-    <t>zinc_copper_ratio_monitoring</t>
-  </si>
-  <si>
-    <t>Zinc citrate ~25 mg elemental included; copper precautionarily excluded. If zinc supplementation continues beyond 3 months, practitioner may wish to monitor copper status.</t>
-  </si>
-  <si>
-    <t>moderate</t>
-  </si>
-  <si>
-    <t>berberine_glucose_and_pregnancy</t>
-  </si>
-  <si>
-    <t>Berberine contraindicated in pregnancy; additive effect with glucose-lowering medications; CYP3A4/CYP2D6 interaction potential.</t>
+    <t>not_applicable</t>
+  </si>
+  <si>
+    <t>iodine_thyroid_antibody_status_not_provided</t>
+  </si>
+  <si>
+    <t>Iodine was not included in this formulation; antibody status not relevant for this submission.</t>
+  </si>
+  <si>
+    <t>applied</t>
+  </si>
+  <si>
+    <t>selenium_red_cell_status_not_provided</t>
+  </si>
+  <si>
+    <t>Selenium omitted in the absence of red-cell selenium data — system safety floor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selenium
+(Selenomethionine)</t>
+  </si>
+  <si>
+    <t>copper_status_not_provided</t>
+  </si>
+  <si>
+    <t>Copper omitted in the absence of Cu:Zn status data — system safety floor.</t>
+  </si>
+  <si>
+    <t>Copper gluconate</t>
+  </si>
+  <si>
+    <t>iron_studies_not_provided</t>
+  </si>
+  <si>
+    <t>Iron omitted — no panel signal of deficiency and no iron studies supplied.</t>
+  </si>
+  <si>
+    <t>Iron bisglycinate</t>
+  </si>
+  <si>
+    <t>age_over_50_female</t>
+  </si>
+  <si>
+    <t>Patient age 56 — within standard adult dosing; no soft escalation triggered (under 75).</t>
   </si>
   <si>
     <t/>
@@ -503,13 +492,13 @@
     <t>Pod budget utilisation</t>
   </si>
   <si>
-    <t>89.0%</t>
+    <t>95.5%</t>
   </si>
   <si>
     <t>Pod weight (estimated)</t>
   </si>
   <si>
-    <t>12,298 mg</t>
+    <t>13,015 mg</t>
   </si>
   <si>
     <t>Ingredients in pod</t>
@@ -539,22 +528,25 @@
     <t>Granules allocated</t>
   </si>
   <si>
+    <t>Antioxidant / Redox (primary)</t>
+  </si>
+  <si>
+    <t>Heavy Metal Detox (primary)</t>
+  </si>
+  <si>
     <t>Anti-inflammatory Core (primary)</t>
   </si>
   <si>
-    <t>Antioxidant / Redox (primary)</t>
-  </si>
-  <si>
     <t>Mitochondrial / Cardiovascular (primary)</t>
   </si>
   <si>
     <t>B-Vitamins / Methylation (secondary)</t>
   </si>
   <si>
-    <t>Gastrointestinal (secondary)</t>
-  </si>
-  <si>
-    <t>Minerals (supportive)</t>
+    <t>Minerals (secondary)</t>
+  </si>
+  <si>
+    <t>Vitamin D / C / Neurotransmitter (supportive)</t>
   </si>
   <si>
     <t>Plan total</t>
@@ -564,7 +556,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -579,12 +571,6 @@
       <name val="Roboto"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Roboto"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFC3AF88"/>
       <sz val="10"/>
       <name val="Roboto"/>
     </font>
@@ -655,7 +641,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -672,23 +658,17 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -701,8 +681,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1044,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1108,7 +1088,7 @@
         <v>13</v>
       </c>
       <c r="E2" s="3">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>14</v>
@@ -1137,83 +1117,83 @@
         <v>21</v>
       </c>
       <c r="C3" s="5">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="5">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" s="3">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E4" s="3">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="5">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E5" s="5">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>14</v>
@@ -1222,36 +1202,36 @@
         <v>15</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" s="3">
-        <v>600</v>
+        <v>150</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="3">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>15</v>
@@ -1277,63 +1257,63 @@
         <v>46</v>
       </c>
       <c r="C7" s="5">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="5">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C8" s="3">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="3">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>56</v>
@@ -1347,39 +1327,39 @@
         <v>58</v>
       </c>
       <c r="C9" s="5">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E9" s="5">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="J9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C10" s="3">
         <v>100</v>
@@ -1391,30 +1371,30 @@
         <v>100</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C11" s="5">
         <v>150</v>
@@ -1426,267 +1406,232 @@
         <v>30</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="K11" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="3">
+        <v>500</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C12" s="3">
-        <v>15</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="E12" s="3">
         <v>2</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="K12" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C13" s="5">
-        <v>500</v>
+        <v>547</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E13" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C14" s="3">
-        <v>20</v>
+        <v>23.52</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="K14" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C15" s="5">
-        <v>520</v>
+        <v>50</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="E15" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="I15" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="4" t="s">
         <v>98</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C16" s="3">
-        <v>500</v>
+        <v>855</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="3">
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="K16" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C17" s="5">
+        <v>25</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C17" s="5">
-        <v>200</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" s="5">
-        <v>20</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H17" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="J17" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="K17" s="4" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="3">
-        <v>77.88</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" s="3">
-        <v>13</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1697,7 +1642,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1707,46 +1652,35 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1767,57 +1701,57 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1828,7 +1762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1839,72 +1773,100 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="D2" s="2" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="C6" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C3" s="4" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>148</v>
+      <c r="D7" s="4" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1915,179 +1877,187 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B5" s="10">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="B6" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="B2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="B5" s="12">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B8" s="12">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+      <c r="B9" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B10" s="12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="B11" s="10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="B8" s="14">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="B12" s="12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="B13" s="10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B10" s="14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="B16" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="B11" s="12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="B17" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="B12" s="14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+      <c r="B18" s="15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="B19" s="16">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B20" s="15">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="B21" s="16">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="B18" s="17">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="B22" s="15">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="B19" s="18">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="B23" s="16">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="B20" s="17">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="B24" s="15">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="B21" s="18">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="B22" s="17">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="B23" s="18">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="B24" s="20">
-        <v>640</v>
+      <c r="B25" s="18">
+        <v>700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add HMP panel class support (EndoSCAN): prompt v0.5.3, first green live-fire 682/710 (96.1%)
</commit_message>
<xml_diff>
--- a/generated-docs/Nof1_FormulationSchedule_SUB-2026-003_DRAFT.xlsx
+++ b/generated-docs/Nof1_FormulationSchedule_SUB-2026-003_DRAFT.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="195">
   <si>
     <t>W Code</t>
   </si>
@@ -50,70 +50,340 @@
     <t>Evidence Pointer</t>
   </si>
   <si>
+    <t>W140019000</t>
+  </si>
+  <si>
+    <t>DIM (3,3'-diindolylmethane)</t>
+  </si>
+  <si>
+    <t>mg</t>
+  </si>
+  <si>
+    <t>Hormone Metabolism</t>
+  </si>
+  <si>
+    <t>STANDARD</t>
+  </si>
+  <si>
+    <t>2-OH Estrone 0.04 ug/gCR (low), 2-OH(E1+E2)/16-OHE1 0.60 (low), Estrogen Quotient 0.24 (low)</t>
+  </si>
+  <si>
+    <t>Foundational hormone_metabolism axis ingredient. Published literature supports DIM as a Phase I CYP1A1 modulator that may shift oestrogen hydroxylation toward the 2-OH pathway — for practitioner consideration given low 2-OH Estrone (0.04 ug/gCR, reference 0.10–1.88) and low 2-OH/16-OH ratio (0.60, reference 1.10–5.60).</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; published literature notes possible mild GI symptoms. The practitioner may wish to monitor and consider clinical correlation.</t>
+  </si>
+  <si>
+    <t>Library entry references for DIM and Phase I oestrogen pathway modulation per published mechanism studies.</t>
+  </si>
+  <si>
+    <t>W040012000</t>
+  </si>
+  <si>
+    <t>Calcium D-glucarate</t>
+  </si>
+  <si>
+    <t>Estrogen Quotient 0.24 (low), 16-OH-dominant pattern</t>
+  </si>
+  <si>
+    <t>Supports glucuronidation pathway and inhibits beta-glucuronidase per published mechanism studies — for practitioner consideration of enterohepatic clearance of conjugated oestrogen metabolites, given low oestrogen quotient.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated. Provides ~80 mg elemental calcium per dose — practitioner may wish to consider in context of total dietary calcium.</t>
+  </si>
+  <si>
+    <t>Library entry references for calcium D-glucarate and glucuronidation/beta-glucuronidase pathway.</t>
+  </si>
+  <si>
+    <t>W010013000</t>
+  </si>
+  <si>
+    <t>Milk thistle (silymarin)</t>
+  </si>
+  <si>
+    <t>Published literature supports silymarin as a Nrf2-mediated Phase II hepatic conjugation supporter — for practitioner consideration of hepatic oestrogen metabolism support.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; the practitioner may wish to consider in context of any liver medications.</t>
+  </si>
+  <si>
+    <t>Library entry references for silymarin and Phase II hepatoprotection.</t>
+  </si>
+  <si>
+    <t>W010019000</t>
+  </si>
+  <si>
+    <t>Resveratrol</t>
+  </si>
+  <si>
+    <t>MODERATE</t>
+  </si>
+  <si>
+    <t>Estrogen Quotient 0.24 (low), 2-OH Estrone (low)</t>
+  </si>
+  <si>
+    <t>Published literature supports resveratrol for mild aromatase modulation and 2-OH pathway support — for practitioner consideration alongside DIM for oestrogen metabolism balance. Dose at Library AUST L limit of 150 mg.</t>
+  </si>
+  <si>
+    <t>TGA-required label warning notes possible interaction with warfarin and other medications. The practitioner may wish to confirm no anticoagulant use before recommending. Not recommended during pregnancy or lactation (not applicable here — adult male).</t>
+  </si>
+  <si>
+    <t>Library entry references for resveratrol mechanism studies and oestrogen pathway modulation.</t>
+  </si>
+  <si>
+    <t>W010003000</t>
+  </si>
+  <si>
+    <t>Ashwagandha</t>
+  </si>
+  <si>
+    <t>Thyroid / Adaptogenic</t>
+  </si>
+  <si>
+    <t>Total 24hr Cortisol 24.91 ug/gCR (low), DHEA in lower portion of range</t>
+  </si>
+  <si>
+    <t>Foundational thyroid_adaptogenic axis ingredient. Published literature including double-blind RCT data supports ashwagandha for HPA resilience and stress modulation — for practitioner consideration given low total urinary cortisol pattern.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated. The practitioner may wish to consider in context of any thyroid medications, immunosuppressants, or sedatives.</t>
+  </si>
+  <si>
+    <t>Library entry references including Salve 2019 (Cureus) and related adaptogen RCTs.</t>
+  </si>
+  <si>
+    <t>W010020000</t>
+  </si>
+  <si>
+    <t>Rhodiola</t>
+  </si>
+  <si>
+    <t>Total 24hr Cortisol 24.91 ug/gCR (low)</t>
+  </si>
+  <si>
+    <t>Published literature supports rhodiola for stress-related fatigue and HPA modulation — complementary adaptogenic support alongside ashwagandha for the HPA-hypocortisolism pattern.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; insomnia possible if dosed late in day. The practitioner may wish to recommend morning dosing.</t>
+  </si>
+  <si>
+    <t>Library entry references including Olsson 2009 and Ishaque 2012 systematic review.</t>
+  </si>
+  <si>
+    <t>W010001000</t>
+  </si>
+  <si>
+    <t>American ginseng (Panax quinquefolius)</t>
+  </si>
+  <si>
+    <t>Published literature including cancer-related fatigue RCTs supports American ginseng as a tonic adaptogen — for practitioner consideration as adjunct to the adaptogen stack for HPA-hypocortisolism.</t>
+  </si>
+  <si>
+    <t>May affect blood pressure and glucose; the practitioner may wish to consider in context of any antihypertensive or glucose-lowering therapy.</t>
+  </si>
+  <si>
+    <t>Library entry references including Barton 2013 N07C2 trial.</t>
+  </si>
+  <si>
+    <t>W030021000</t>
+  </si>
+  <si>
+    <t>Coenzyme Q10</t>
+  </si>
+  <si>
+    <t>Mitochondrial / Cardiovascular</t>
+  </si>
+  <si>
+    <t>Total 24hr Cortisol 24.91 ug/gCR (low) — associated energy/fatigue presentation</t>
+  </si>
+  <si>
+    <t>Published literature supports CoQ10 for mitochondrial bioenergetics — for practitioner consideration given HPA-hypocortisolism pattern and associated fatigue presentation.</t>
+  </si>
+  <si>
+    <t>TGA-required label warning advises caution with warfarin. The practitioner may wish to confirm no anticoagulant use.</t>
+  </si>
+  <si>
+    <t>Library entry references for CoQ10 mitochondrial mechanism studies.</t>
+  </si>
+  <si>
+    <t>W030008000</t>
+  </si>
+  <si>
+    <t>Vitamin B12 (methylcobalamin)</t>
+  </si>
+  <si>
+    <t>mcg</t>
+  </si>
+  <si>
+    <t>B-Vitamins / Methylation</t>
+  </si>
+  <si>
+    <t>Low 2-MeOH Estrone (substrate-limited)</t>
+  </si>
+  <si>
+    <t>Methylation cofactor supporting COMT-mediated methylation of catechol oestrogens — for practitioner consideration alongside DIM (which provides 2-OH substrate).</t>
+  </si>
+  <si>
+    <t>Generally well tolerated.</t>
+  </si>
+  <si>
+    <t>Library entry references for methylcobalamin and methylation cycle.</t>
+  </si>
+  <si>
+    <t>W030027000</t>
+  </si>
+  <si>
+    <t>Folate (as calcium folinate)</t>
+  </si>
+  <si>
+    <t>Methylation cofactor at Library AUST L maximum (delivering 500 mcg folinic acid). Supports COMT methylation and overall methylation cycle.</t>
+  </si>
+  <si>
+    <t>Practitioner-only; B12 status should be assured before high-dose folate to avoid masking B12 deficiency. Combined methylcobalamin in this formulation addresses this consideration.</t>
+  </si>
+  <si>
+    <t>Library entry references for calcium folinate and methylation support.</t>
+  </si>
+  <si>
+    <t>W030012000</t>
+  </si>
+  <si>
+    <t>Vitamin B6 (P5P)</t>
+  </si>
+  <si>
+    <t>Low 2-MeOH Estrone (substrate-limited methylation)</t>
+  </si>
+  <si>
+    <t>Methylation cofactor and neurotransmitter/steroid synthesis cofactor — for practitioner consideration in the HPA and methylation context. Dose deliberately conservative given current TGA-required B6 label warnings about peripheral neuropathy.</t>
+  </si>
+  <si>
+    <t>TGA-required label warning regarding peripheral neuropathy with extended high-dose B6. Dose chosen well below regulatory thresholds.</t>
+  </si>
+  <si>
+    <t>Library entry references for P5P methylation and steroidogenesis support.</t>
+  </si>
+  <si>
+    <t>W030011000</t>
+  </si>
+  <si>
+    <t>Riboflavin (B2)</t>
+  </si>
+  <si>
+    <t>Methylation cycle support</t>
+  </si>
+  <si>
+    <t>FAD/FMN cofactor supporting MTHFR and overall methylation cycle — for practitioner consideration as a methylation cofactor adjunct.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; harmless yellow urine discolouration may occur.</t>
+  </si>
+  <si>
+    <t>Library entry references for riboflavin methylation cofactor role.</t>
+  </si>
+  <si>
+    <t>W030004000</t>
+  </si>
+  <si>
+    <t>Pantothenic acid (B5)</t>
+  </si>
+  <si>
+    <t>B5 is the CoA precursor and a specific adrenal cofactor referenced in the laboratory comment for HPA support — for practitioner consideration given the low total urinary cortisol pattern.</t>
+  </si>
+  <si>
+    <t>Generally very well tolerated.</t>
+  </si>
+  <si>
+    <t>Library entry references for pantothenic acid adrenal cofactor role.</t>
+  </si>
+  <si>
+    <t>W030003000</t>
+  </si>
+  <si>
+    <t>Nicotinamide (B3)</t>
+  </si>
+  <si>
+    <t>General redox/energy support</t>
+  </si>
+  <si>
+    <t>NAD precursor supporting energy and redox metabolism — for practitioner consideration as a baseline B-complex cofactor.</t>
+  </si>
+  <si>
+    <t>Nicotinamide form chosen (rather than niacin) — not associated with flushing.</t>
+  </si>
+  <si>
+    <t>Library entry references for nicotinamide and NAD/redox metabolism.</t>
+  </si>
+  <si>
+    <t>W040002000</t>
+  </si>
+  <si>
+    <t>Magnesium glycinate</t>
+  </si>
+  <si>
+    <t>Minerals</t>
+  </si>
+  <si>
+    <t>Low 2-MeOH metabolites (COMT cofactor support), Total 24hr Cortisol 24.91 ug/gCR (low) — HPA support</t>
+  </si>
+  <si>
+    <t>COMT cofactor and HPA support agent. Dose reduced from clinical target (~300 mg elemental Mg) to ~120 mg elemental to fit pod granule budget — for practitioner consideration the patient may benefit from an additional standalone magnesium dose to reach the full clinical target.</t>
+  </si>
+  <si>
+    <t>Generally very well tolerated at this dose; the glycinate form has the lowest osmotic laxative effect.</t>
+  </si>
+  <si>
+    <t>Library entry references for magnesium glycinate, COMT cofactor function, and HPA support.</t>
+  </si>
+  <si>
+    <t>W040008000</t>
+  </si>
+  <si>
+    <t>Zinc citrate</t>
+  </si>
+  <si>
+    <t>Hormone_metabolism axis adjunct, General immune/steroidogenic support</t>
+  </si>
+  <si>
+    <t>Aromatase modulation cofactor and supports steroidogenesis and immune function — moderate dose (~25 mg elemental) chosen deliberately rather than maximum given testosterone is mid-range and androgen-excess pattern is not active.</t>
+  </si>
+  <si>
+    <t>Long-term use of zinc above 25 mg elemental may warrant copper status monitoring per published frameworks. The practitioner may wish to consider copper status at follow-up if used long-term.</t>
+  </si>
+  <si>
+    <t>Library entry references for zinc and aromatase/steroidogenesis modulation.</t>
+  </si>
+  <si>
     <t>W140010000</t>
   </si>
   <si>
     <t>N-acetyl cysteine (NAC)</t>
   </si>
   <si>
-    <t>mg</t>
-  </si>
-  <si>
     <t>Antioxidant / Redox</t>
   </si>
   <si>
-    <t>STANDARD</t>
-  </si>
-  <si>
-    <t>8-OHdG 3.80, Pyroglutamic 28.8, t,t-Muconic 0.20</t>
-  </si>
-  <si>
-    <t>Glutathione precursor supporting xenobiotic conjugation and antioxidant defence; addresses 8-OHdG 3.80 (&lt;2.70), pyroglutamic acid at upper range, and the xenobiotic burden pattern (t,t-muconic, 3-methylhippuric).</t>
-  </si>
-  <si>
-    <t>Standard contraindication checks: medications not listed in submission; NAC is generally well tolerated.</t>
-  </si>
-  <si>
-    <t>Published evidence supports NAC for glutathione repletion and antioxidant support; clinical relevance for this patient is for practitioner assessment.</t>
-  </si>
-  <si>
-    <t>W010013000</t>
-  </si>
-  <si>
-    <t>Milk thistle (silymarin)</t>
-  </si>
-  <si>
-    <t>Heavy Metal Detox</t>
-  </si>
-  <si>
-    <t>t,t-Muconic 0.20, 5-HMF 18.5, Benzoic 25.0</t>
-  </si>
-  <si>
-    <t>Nrf2-mediated Phase II upregulation and hepatoprotection; addresses xenobiotic-burdened pattern (t,t-muconic, 3-methylhippuric, 4-HBA, 5-HMF).</t>
-  </si>
-  <si>
-    <t>Generally well tolerated.</t>
-  </si>
-  <si>
-    <t>Published mechanism and clinical literature supports milk thistle as hepatic/Phase II support — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W040012000</t>
-  </si>
-  <si>
-    <t>Calcium D-glucarate</t>
-  </si>
-  <si>
-    <t>4-HBA 0.64, 5-HMF 18.5, Benzoic 25.0</t>
-  </si>
-  <si>
-    <t>Glucuronidation support via beta-glucuronidase inhibition; addresses paraben/phthalate/xenobiotic conjugation load.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; phthalate marker within range but paraben (4-HBA) elevated.</t>
-  </si>
-  <si>
-    <t>Published mechanism literature supports Cal D-glucarate for Phase II glucuronidation — practitioner to assess.</t>
+    <t>Antioxidant buffer for catechol oestrogen metabolism</t>
+  </si>
+  <si>
+    <t>Glutathione precursor and quinone-quenching agent for catechol-oestrogen metabolism — for practitioner consideration as antioxidant support in the oestrogen metabolism context.</t>
+  </si>
+  <si>
+    <t>Library entry references for NAC and glutathione cycling.</t>
+  </si>
+  <si>
+    <t>W010031000</t>
+  </si>
+  <si>
+    <t>Quercetin</t>
+  </si>
+  <si>
+    <t>Flavonoid antioxidant with published mechanism studies for CYP1B1 modulation and antioxidant support — for practitioner consideration as complementary antioxidant in the oestrogen metabolism context.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; may have mild CYP interactions per published literature.</t>
+  </si>
+  <si>
+    <t>Library entry references for quercetin antioxidant and CYP modulation.</t>
   </si>
   <si>
     <t>W030001000</t>
@@ -122,217 +392,19 @@
     <t>Vitamin C (ascorbic acid)</t>
   </si>
   <si>
-    <t>8-OHdG 3.80</t>
-  </si>
-  <si>
-    <t>Antioxidant defence aligned with elevated 8-OHdG and broad xenobiotic redox demand.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; consider divided doses if GI tolerability is an issue.</t>
-  </si>
-  <si>
-    <t>Published evidence supports vitamin C as a water-soluble antioxidant — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W010019000</t>
-  </si>
-  <si>
-    <t>Resveratrol</t>
-  </si>
-  <si>
-    <t>8-OHdG 3.80, LTE4 195</t>
-  </si>
-  <si>
-    <t>Nrf2/sirtuin antioxidant support complementing NAC and vitamin C for the oxidative stress pattern.</t>
-  </si>
-  <si>
-    <t>Anticoagulant interaction theoretical; practitioner to review medications.</t>
-  </si>
-  <si>
-    <t>Published RCT and mechanism literature for antioxidant/anti-inflammatory effects — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W010029000</t>
-  </si>
-  <si>
-    <t>Turmeric (curcumin)</t>
-  </si>
-  <si>
-    <t>Anti-inflammatory Core</t>
-  </si>
-  <si>
-    <t>LTE4 195, Quinolinic 11.8</t>
-  </si>
-  <si>
-    <t>NF-κB anchor for inflammatory load (LTE4 elevation, kynurenine inflammatory shift).</t>
-  </si>
-  <si>
-    <t>Caution with anticoagulants; standard contraindication checks.</t>
-  </si>
-  <si>
-    <t>RCT evidence supports curcumin's anti-inflammatory mechanism — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W010022000</t>
-  </si>
-  <si>
-    <t>Boswellia serrata</t>
-  </si>
-  <si>
-    <t>LTE4 195</t>
-  </si>
-  <si>
-    <t>5-LOX inhibition specifically relevant to elevated leukotriene E4. Dose trimmed for pod budget; clinical target 800 mg may be considered as additional standalone if indicated.</t>
-  </si>
-  <si>
-    <t>Published evidence for 5-LOX-pathway modulation — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W010031000</t>
-  </si>
-  <si>
-    <t>Quercetin</t>
-  </si>
-  <si>
-    <t>Mast-cell stabilising and adjunctive anti-inflammatory action complementing LTE4-driven inflammation.</t>
-  </si>
-  <si>
-    <t>Published mechanism literature for mast-cell modulation — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W030021000</t>
-  </si>
-  <si>
-    <t>Coenzyme Q10</t>
-  </si>
-  <si>
-    <t>Mitochondrial / Cardiovascular</t>
-  </si>
-  <si>
-    <t>3-MGA 6.32, Mevalonolactone 2.80, Isocitrate 86, 2-OG 65</t>
-  </si>
-  <si>
-    <t>Mitochondrial electron transport and mevalonate pathway support; addresses 3-MGA, mevalonolactone, and TCA cycle markers.</t>
-  </si>
-  <si>
-    <t>Standard interaction note with warfarin.</t>
-  </si>
-  <si>
-    <t>Published cardiology/mitochondrial literature — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W030020000</t>
-  </si>
-  <si>
-    <t>Alpha-lipoic acid</t>
-  </si>
-  <si>
-    <t>2-OG 65, Isocitrate 86, 8-OHdG 3.80</t>
-  </si>
-  <si>
-    <t>Cofactor for 2-OG dehydrogenase and pyruvate dehydrogenase; addresses 2-OG and isocitrate elevation and contributes to antioxidant defence.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; mild hypoglycaemic effect possible.</t>
-  </si>
-  <si>
-    <t>Published mechanism literature — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W030008000</t>
-  </si>
-  <si>
-    <t>Methylcobalamin (B12)</t>
-  </si>
-  <si>
-    <t>mcg</t>
-  </si>
-  <si>
-    <t>B-Vitamins / Methylation</t>
-  </si>
-  <si>
-    <t>Guanidinoacetic 4.80, KMBA 3.20, 5-Methylcytosine 68</t>
-  </si>
-  <si>
-    <t>Methylation cycle support addressing methyl-acceptor demand (guanidinoacetic, KMBA, 5-methylcytosine).</t>
-  </si>
-  <si>
-    <t>Standard B12 considerations.</t>
-  </si>
-  <si>
-    <t>Published methylation literature — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W030027000</t>
-  </si>
-  <si>
-    <t>Calcium folinate</t>
-  </si>
-  <si>
-    <t>Guanidinoacetic 4.80, 5-Methylcytosine 68</t>
-  </si>
-  <si>
-    <t>Folate cycle cofactor for one-carbon metabolism; supports the methylation demand pattern.</t>
-  </si>
-  <si>
-    <t>May mask B12 deficiency in megaloblastic anaemia — B12 included concurrently.</t>
-  </si>
-  <si>
-    <t>W030012000</t>
-  </si>
-  <si>
-    <t>Pyridoxal-5-phosphate (P5P / active B6)</t>
-  </si>
-  <si>
-    <t>Xanthurenic 1.92, Quinolinic 11.8, Kynurenic 3.10</t>
-  </si>
-  <si>
-    <t>Active B6 anchoring kynurenine pathway support given xanthurenic 1.92 (&lt;0.96) and quinolinic 11.8 (&lt;9.10); B6 cofactor for kynureninase.</t>
-  </si>
-  <si>
-    <t>TGA advises stopping if tingling/numbness occurs; dose kept conservative.</t>
-  </si>
-  <si>
-    <t>Published kynurenine pathway literature — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W030011000</t>
-  </si>
-  <si>
-    <t>Riboflavin (B2)</t>
-  </si>
-  <si>
-    <t>2-OG 65, Kynurenic 3.10</t>
-  </si>
-  <si>
-    <t>FAD cofactor for mitochondrial flavoproteins and kynurenine monooxygenase; supports both TCA strain and kynurenine pattern.</t>
-  </si>
-  <si>
-    <t>Generally well tolerated; yellow urine expected.</t>
-  </si>
-  <si>
-    <t>Published B2 metabolism literature — practitioner to assess.</t>
-  </si>
-  <si>
-    <t>W040002000</t>
-  </si>
-  <si>
-    <t>Magnesium glycinate</t>
-  </si>
-  <si>
-    <t>Minerals</t>
-  </si>
-  <si>
-    <t>2-OG 65, Isocitrate 86, Guanidinoacetic 4.80</t>
-  </si>
-  <si>
-    <t>Broad mitochondrial/methylation cofactor at conservative in-pod elemental dose (100 mg). The glycinate carrier also contributes glycine equivalents incidentally supportive of conjugation pathways. Practitioner may wish to consider additional standalone magnesium toward a clinical target if symptomatically indicated.</t>
-  </si>
-  <si>
-    <t>Standard renal considerations.</t>
-  </si>
-  <si>
-    <t>Published magnesium clinical literature — practitioner to assess.</t>
+    <t>Vitamin D / C / Neurotransmitter</t>
+  </si>
+  <si>
+    <t>Total 24hr Cortisol 24.91 ug/gCR (low) — adrenal cofactor</t>
+  </si>
+  <si>
+    <t>Adrenal cofactor specifically referenced in the laboratory comment as supportive in HPA-hypocortisolism, alongside antioxidant function.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated; high doses may cause GI upset.</t>
+  </si>
+  <si>
+    <t>Library entry references for vitamin C and adrenal/antioxidant function.</t>
   </si>
   <si>
     <t>W030005000</t>
@@ -341,19 +413,16 @@
     <t>Vitamin D3 (cholecalciferol)</t>
   </si>
   <si>
-    <t>Vitamin D / C / Neurotransmitter</t>
-  </si>
-  <si>
-    <t>General repletion</t>
-  </si>
-  <si>
-    <t>Conservative repletion dose at AUST L cap (25 mcg = 1000 IU); supports general immune/redox status. 25-OH D not measured on this panel.</t>
-  </si>
-  <si>
-    <t>Practitioner may wish to assess serum 25-OH D to guide longer-term dosing.</t>
-  </si>
-  <si>
-    <t>Published vitamin D supplementation literature — practitioner to assess.</t>
+    <t>General endocrine support</t>
+  </si>
+  <si>
+    <t>General endocrine support at Library AUST L maximum (1000 IU). Published literature supports vitamin D adequacy as relevant to overall endocrine and immune function.</t>
+  </si>
+  <si>
+    <t>Generally well tolerated at this dose. The practitioner may wish to confirm 25-OH vitamin D status if not recently assessed.</t>
+  </si>
+  <si>
+    <t>Library entry references for vitamin D3.</t>
   </si>
   <si>
     <t>Adjustment Type</t>
@@ -365,16 +434,25 @@
     <t>Affected Ingredient(s)</t>
   </si>
   <si>
-    <t>in_pod_dose_below_clinical_target</t>
-  </si>
-  <si>
-    <t>Boswellia in-pod dose 300 mg vs clinical target 800 mg — trimmed for pod budget. Practitioner may consider standalone top-up.</t>
-  </si>
-  <si>
-    <t>Boswellia (Frankincense)</t>
-  </si>
-  <si>
-    <t>Magnesium glycinate in-pod elemental 100 mg vs broader clinical target — split-dosing may be considered.</t>
+    <t>Dose reduced for pod budget</t>
+  </si>
+  <si>
+    <t>Magnesium glycinate proposed at 1023.5 mg salt (delivering ~120 mg elemental Mg), reduced from a clinical target of ~300 mg elemental Mg (~2562 mg salt) due to pod granule budget constraints. The practitioner may wish to consider an additional standalone magnesium dose if the patient benefits from the higher target.</t>
+  </si>
+  <si>
+    <t>Conservative dose by clinical choice</t>
+  </si>
+  <si>
+    <t>Zinc citrate proposed at ~25 mg elemental rather than the Library maximum of 50 mg elemental — deliberately conservative given testosterone is mid-range and androgen-excess pattern is not active. The practitioner may wish to adjust based on copper:zinc considerations and clinical correlation.</t>
+  </si>
+  <si>
+    <t>Regulatory cap</t>
+  </si>
+  <si>
+    <t>Calcium folinate dosed at Library AUST L maximum of 547 mcg salt (500 mcg folinic acid). Resveratrol dosed at Library AUST L maximum of 150 mg. Vitamin D3 dosed at Library AUST L maximum of 25 mcg (1000 IU). Vitamin B6 dosed conservatively at 10 mg elemental given TGA-required peripheral neuropathy label warnings for higher doses.</t>
+  </si>
+  <si>
+    <t>Calcium folinate, Resveratrol, Vitamin D3, Vitamin B6 (P5P)</t>
   </si>
   <si>
     <t>Recommendation</t>
@@ -386,31 +464,13 @@
     <t>Practitioner Note</t>
   </si>
   <si>
-    <t>Glycine 1.5–3 g daily</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Glycine is the canonical Phase II conjugator for benzoate, xylene/toluene metabolites and HMF-derived furancarbonyl conjugates. Given elevated benzoic acid, 3-methylhippuric, 4-HBA and furancarbonylglycine, the practitioner may wish to consider glycine repletion alongside the in-pod conjugation support. Not in current Library as a granule ingredient.</t>
-  </si>
-  <si>
-    <t>EPA/DHA omega-3 fish oil 2–3 g daily</t>
-  </si>
-  <si>
-    <t>Given leukotriene E4 elevation (195 vs &lt;100), the practitioner may wish to consider an EPA-predominant omega-3 to shift eicosanoid balance. Not in current granule Library.</t>
-  </si>
-  <si>
-    <t>L-carnitine 1–2 g daily</t>
-  </si>
-  <si>
-    <t>Given mild adipic acid elevation suggesting omega-oxidation when beta-oxidation is constrained, the practitioner may wish to consider carnitine support. Not in current Library.</t>
-  </si>
-  <si>
-    <t>Multi-strain probiotic (Lactobacillus / Bifidobacterium spp.) 20–40 billion CFU daily</t>
-  </si>
-  <si>
-    <t>Given modest dysbiosis markers (arabinose, 3,4-DHBA, 3-HPAA), the practitioner may wish to consider probiotic support and dietary review. Not in current granule Library.</t>
+    <t>(none)</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>No standalone recommendations or pod exclusions on this formulation.</t>
   </si>
   <si>
     <t>Severity</t>
@@ -422,59 +482,49 @@
     <t>informational</t>
   </si>
   <si>
-    <t>no_medication_list_provided</t>
-  </si>
-  <si>
-    <t>Clinical notes did not list current medications. Standard contraindication screens (5-HTP with serotonergics; berberine with glucose-lowering agents; curcumin/resveratrol with anticoagulants; magnesium with antibiotics/bisphosphonates; St John's Wort with multiple meds) were therefore applied to the formulation in the abstract. 5-HTP and berberine were not included in this formulation. Curcumin, resveratrol and magnesium have been included — practitioner to verify against the patient's full medication list.</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>not_applicable</t>
-  </si>
-  <si>
-    <t>iodine_thyroid_antibody_status_not_provided</t>
-  </si>
-  <si>
-    <t>Iodine was not included in this formulation; antibody status not relevant for this submission.</t>
+    <t>No medication context provided</t>
+  </si>
+  <si>
+    <t>Practitioner's clinical notes did not list current medications. Standard contraindication checks are therefore based on the formulation alone. The practitioner may wish to confirm absence of: anticoagulants (relevant to resveratrol and CoQ10 per TGA warnings), thyroid medications (relevant to ashwagandha caution), immunosuppressants (relevant to adaptogens), glucose-lowering agents (relevant to American ginseng), antihypertensives (relevant to American ginseng), and CYP3A4/2D6 substrates.</t>
+  </si>
+  <si>
+    <t>moderate</t>
+  </si>
+  <si>
+    <t>Resveratrol — warfarin interaction risk</t>
+  </si>
+  <si>
+    <t>TGA-required label warning notes resveratrol may affect anticoagulants including warfarin. Confirm patient is not on anticoagulants before recommending.</t>
+  </si>
+  <si>
+    <t>CoQ10 — warfarin interaction risk</t>
+  </si>
+  <si>
+    <t>TGA-required label warning notes caution with warfarin therapy. Confirm patient is not on anticoagulants before recommending.</t>
+  </si>
+  <si>
+    <t>monitor</t>
+  </si>
+  <si>
+    <t>Vitamin B6 peripheral neuropathy</t>
+  </si>
+  <si>
+    <t>TGA-required label warning advises monitoring for tingling, burning, or numbness with vitamin B6 use. Dose in this formulation is conservative (10 mg pyridoxine equivalent) and well below regulatory thresholds, but the practitioner may wish to monitor on follow-up.</t>
+  </si>
+  <si>
+    <t>Long-term zinc and copper status</t>
+  </si>
+  <si>
+    <t>Zinc at 25 mg elemental long-term (&gt;3 months) warrants practitioner consideration of copper status per standard frameworks. Re-test or clinical review at appropriate intervals.</t>
   </si>
   <si>
     <t>applied</t>
   </si>
   <si>
-    <t>selenium_red_cell_status_not_provided</t>
-  </si>
-  <si>
-    <t>Selenium omitted in the absence of red-cell selenium data — system safety floor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selenium
-(Selenomethionine)</t>
-  </si>
-  <si>
-    <t>copper_status_not_provided</t>
-  </si>
-  <si>
-    <t>Copper omitted in the absence of Cu:Zn status data — system safety floor.</t>
-  </si>
-  <si>
-    <t>Copper gluconate</t>
-  </si>
-  <si>
-    <t>iron_studies_not_provided</t>
-  </si>
-  <si>
-    <t>Iron omitted — no panel signal of deficiency and no iron studies supplied.</t>
-  </si>
-  <si>
-    <t>Iron bisglycinate</t>
-  </si>
-  <si>
-    <t>age_over_50_female</t>
-  </si>
-  <si>
-    <t>Patient age 56 — within standard adult dosing; no soft escalation triggered (under 75).</t>
+    <t>Iodine — binding exclusion applied</t>
+  </si>
+  <si>
+    <t>Iodine above 150 mcg not included given absence of thyroid antibody data on this panel. No iodine included in formulation as no thyroid driver is activated.</t>
   </si>
   <si>
     <t/>
@@ -492,13 +542,13 @@
     <t>Pod budget utilisation</t>
   </si>
   <si>
-    <t>95.5%</t>
+    <t>96.1%</t>
   </si>
   <si>
     <t>Pod weight (estimated)</t>
   </si>
   <si>
-    <t>13,015 mg</t>
+    <t>13,101 mg</t>
   </si>
   <si>
     <t>Ingredients in pod</t>
@@ -528,19 +578,19 @@
     <t>Granules allocated</t>
   </si>
   <si>
-    <t>Antioxidant / Redox (primary)</t>
-  </si>
-  <si>
-    <t>Heavy Metal Detox (primary)</t>
-  </si>
-  <si>
-    <t>Anti-inflammatory Core (primary)</t>
-  </si>
-  <si>
-    <t>Mitochondrial / Cardiovascular (primary)</t>
+    <t>Hormone Metabolism (primary)</t>
+  </si>
+  <si>
+    <t>Thyroid / Adaptogenic (primary)</t>
   </si>
   <si>
     <t>B-Vitamins / Methylation (secondary)</t>
+  </si>
+  <si>
+    <t>Mitochondrial / Cardiovascular (secondary)</t>
+  </si>
+  <si>
+    <t>Antioxidant / Redox (secondary)</t>
   </si>
   <si>
     <t>Minerals (secondary)</t>
@@ -556,7 +606,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -571,6 +621,18 @@
       <name val="Roboto"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF666666"/>
+      <sz val="10"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFC3AF88"/>
       <sz val="10"/>
       <name val="Roboto"/>
     </font>
@@ -641,7 +703,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -658,17 +720,24 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -681,8 +750,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1024,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1082,13 +1151,13 @@
         <v>12</v>
       </c>
       <c r="C2" s="3">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E2" s="3">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>14</v>
@@ -1117,121 +1186,121 @@
         <v>21</v>
       </c>
       <c r="C3" s="5">
-        <v>150</v>
+        <v>500</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="5">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="C4" s="3">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E4" s="3">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C5" s="5">
-        <v>500</v>
+        <v>150</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E5" s="5">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>14</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="H5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="C6" s="3">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="3">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>15</v>
@@ -1257,194 +1326,194 @@
         <v>46</v>
       </c>
       <c r="C7" s="5">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="5">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="C8" s="3">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="3">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C9" s="5">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>13</v>
       </c>
       <c r="E9" s="5">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C10" s="3">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="E10" s="3">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C11" s="5">
-        <v>150</v>
+        <v>547</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="E11" s="5">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C12" s="3">
-        <v>500</v>
+        <v>15.68</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="E12" s="3">
         <v>2</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>78</v>
@@ -1467,16 +1536,16 @@
         <v>83</v>
       </c>
       <c r="C13" s="5">
-        <v>547</v>
+        <v>20</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="E13" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>15</v>
@@ -1491,33 +1560,33 @@
         <v>86</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C14" s="3">
-        <v>23.52</v>
+        <v>218.4</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="3">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>90</v>
@@ -1546,7 +1615,7 @@
         <v>5</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>15</v>
@@ -1572,13 +1641,13 @@
         <v>100</v>
       </c>
       <c r="C16" s="3">
-        <v>855</v>
+        <v>1023.5</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="3">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>101</v>
@@ -1607,31 +1676,171 @@
         <v>107</v>
       </c>
       <c r="C17" s="5">
-        <v>25</v>
+        <v>77.62</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="E17" s="5">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="G17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H17" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="J17" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="K17" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="K17" s="4" t="s">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>112</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="3">
+        <v>500</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="3">
+        <v>100</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="5">
+        <v>250</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="5">
+        <v>23</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C20" s="3">
+        <v>500</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="3">
+        <v>50</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C21" s="5">
+        <v>25</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" s="5">
+        <v>2</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1642,7 +1851,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1652,35 +1861,46 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>100</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -1691,7 +1911,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1701,57 +1921,24 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>147</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>131</v>
+      <c r="A2" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -1773,100 +1960,100 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>138</v>
+      <c r="A3" s="7" t="s">
+        <v>157</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>137</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>141</v>
+      <c r="A4" s="8" t="s">
+        <v>157</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>144</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>141</v>
+      <c r="A5" s="7" t="s">
+        <v>162</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>147</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>141</v>
+      <c r="A6" s="8" t="s">
+        <v>162</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>150</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1886,178 +2073,178 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="B1" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>154</v>
+      <c r="A2" s="9" t="s">
+        <v>171</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>153</v>
+      <c r="A4" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="B5" s="10">
-        <v>678</v>
+      <c r="A5" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" s="13">
+        <v>682</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>158</v>
+      <c r="A6" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>160</v>
+      <c r="A7" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="B8" s="12">
-        <v>16</v>
+      <c r="A8" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B8" s="15">
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="B9" s="10">
+      <c r="A9" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B9" s="13">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="B10" s="12">
-        <v>4</v>
+      <c r="A10" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B10" s="15">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="B11" s="10">
+      <c r="A11" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="B11" s="13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" s="15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B13" s="13">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="B12" s="12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="B13" s="10">
-        <v>6</v>
-      </c>
-    </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>153</v>
+      <c r="A16" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>169</v>
+      <c r="A17" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="B18" s="15">
-        <v>150</v>
+      <c r="A18" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B18" s="18">
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B19" s="16">
+      <c r="A19" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B19" s="19">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" s="18">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" s="19">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" s="18">
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="B20" s="15">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="B21" s="16">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="B22" s="15">
-        <v>85</v>
-      </c>
-    </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="B23" s="16">
-        <v>35</v>
+      <c r="A23" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" s="19">
+        <v>145</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="B24" s="15">
-        <v>30</v>
+      <c r="A24" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="18">
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="B25" s="18">
-        <v>700</v>
+      <c r="A25" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" s="21">
+        <v>780</v>
       </c>
     </row>
   </sheetData>

</xml_diff>